<commit_message>
Actualización automática - 2026-03-27 07:59:58
</commit_message>
<xml_diff>
--- a/CS_AMONSTACIONES Y ASISTENCIAS.xlsx
+++ b/CS_AMONSTACIONES Y ASISTENCIAS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge Vasquez\Ranking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD4F311-8A97-4774-B771-B284FD1E1883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{392F5F4D-7C3D-4252-9388-D297E511821D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{5713294A-7509-40D5-8A83-45B119F81220}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{5713294A-7509-40D5-8A83-45B119F81220}"/>
   </bookViews>
   <sheets>
     <sheet name="TARDANZA" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="68">
   <si>
     <t>SUPERVISOR</t>
   </si>
@@ -88,9 +88,6 @@
   </si>
   <si>
     <t>MARZO_2026</t>
-  </si>
-  <si>
-    <t>CANT</t>
   </si>
   <si>
     <t>LUCERO JORDAN</t>
@@ -567,6 +564,18 @@
   </si>
   <si>
     <t>CONDICION</t>
+  </si>
+  <si>
+    <t>DIAS</t>
+  </si>
+  <si>
+    <t>LEONOR NAVARRO</t>
+  </si>
+  <si>
+    <t>CALL</t>
+  </si>
+  <si>
+    <t>03, 04, 05, 11, 17, 18, 19, 20, 23, 24</t>
   </si>
 </sst>
 </file>
@@ -661,47 +670,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -725,16 +694,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0DF93EC0-0CD6-4D6A-AB03-F558AB25C52A}" name="Tabla1" displayName="Tabla1" ref="A1:I11" totalsRowShown="0">
-  <autoFilter ref="A1:I11" xr:uid="{0DF93EC0-0CD6-4D6A-AB03-F558AB25C52A}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0DF93EC0-0CD6-4D6A-AB03-F558AB25C52A}" name="Tabla1" displayName="Tabla1" ref="A1:G12" totalsRowShown="0">
+  <autoFilter ref="A1:G12" xr:uid="{0DF93EC0-0CD6-4D6A-AB03-F558AB25C52A}"/>
+  <tableColumns count="7">
     <tableColumn id="7" xr3:uid="{2D87A607-9992-4097-BE7F-1614E56B0873}" name="MES"/>
     <tableColumn id="1" xr3:uid="{1294BCC6-BEEB-4094-B6C3-2197DD6C8D40}" name="ASESOR"/>
     <tableColumn id="9" xr3:uid="{47D831E0-5DE9-40B2-BC54-C325F5203DD7}" name="CONDICION"/>
-    <tableColumn id="2" xr3:uid="{AB10FB53-6211-4E17-94C8-6862A8A822F0}" name="DNI"/>
     <tableColumn id="3" xr3:uid="{49578531-FCCA-44BA-A89C-9805E84215A6}" name="AMONESTACIÓN"/>
-    <tableColumn id="4" xr3:uid="{98E68532-1529-46E4-A484-87800564F29B}" name="CANT"/>
-    <tableColumn id="5" xr3:uid="{1571C9AB-E209-4F68-8491-8C613C34B2FF}" name="DÍA" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{1571C9AB-E209-4F68-8491-8C613C34B2FF}" name="DIAS" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{64615F66-6C41-4881-9DF9-E5F7029B80E6}" name="SUPERVISOR"/>
     <tableColumn id="8" xr3:uid="{9EE7AAE5-10AE-4A9D-84AF-72FA9F56DF8B}" name="MEMOS"/>
   </tableColumns>
@@ -743,16 +710,14 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4621A63B-45B4-4A84-9317-F04F20244068}" name="Tabla2" displayName="Tabla2" ref="A1:I7" totalsRowShown="0">
-  <autoFilter ref="A1:I7" xr:uid="{4621A63B-45B4-4A84-9317-F04F20244068}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4621A63B-45B4-4A84-9317-F04F20244068}" name="Tabla2" displayName="Tabla2" ref="A1:G7" totalsRowShown="0">
+  <autoFilter ref="A1:G7" xr:uid="{4621A63B-45B4-4A84-9317-F04F20244068}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{556029B8-BA77-4441-953E-47C9680421B4}" name="MES"/>
     <tableColumn id="2" xr3:uid="{4E2D1AC5-4A1E-4437-AF5B-423CD1A45581}" name="ASESOR"/>
     <tableColumn id="9" xr3:uid="{A4A5ED6C-152F-4277-8E84-110829762638}" name="CONDICION"/>
-    <tableColumn id="3" xr3:uid="{A91D9530-235B-4519-A64B-659A2201B8F5}" name="DNI"/>
     <tableColumn id="4" xr3:uid="{58340943-27A3-4CF0-996E-C6E2C960D309}" name="AMONESTACIÓN"/>
-    <tableColumn id="5" xr3:uid="{D72F5082-6701-40DF-81E3-83FC1A3DDF45}" name="CANT"/>
-    <tableColumn id="6" xr3:uid="{8828FFCB-5586-4AB9-8B34-E9BC1C1CE0E9}" name="DÍA" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{8828FFCB-5586-4AB9-8B34-E9BC1C1CE0E9}" name="DIAS" dataDxfId="1"/>
     <tableColumn id="7" xr3:uid="{80C78F9C-B714-4B80-96B9-A8AA1049FAFC}" name="SUPERVISOR"/>
     <tableColumn id="8" xr3:uid="{A6556496-72E6-4FEE-873A-AC9005D3F82A}" name="MEMOS"/>
   </tableColumns>
@@ -767,7 +732,7 @@
     <tableColumn id="1" xr3:uid="{E561B0E1-16FD-472B-A64B-7F88DBD86D09}" name="MES"/>
     <tableColumn id="2" xr3:uid="{D58CEE17-F4EC-4B53-B6C7-243438D5B993}" name="ASESOR"/>
     <tableColumn id="3" xr3:uid="{93DC7A31-27F7-4F77-8810-1C5A6F7FA80B}" name="DNI"/>
-    <tableColumn id="4" xr3:uid="{4C6B1EBB-E59E-441D-ADC9-05C1804745DC}" name="DÍA" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{4C6B1EBB-E59E-441D-ADC9-05C1804745DC}" name="DÍA" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{CB80CF62-8766-4CF2-B8D6-E7EC5526FE52}" name="MOTIVO"/>
     <tableColumn id="6" xr3:uid="{1C552CAB-0DF6-4B1D-83CC-7D8ABCDD76A9}" name="SUPERVISOR"/>
   </tableColumns>
@@ -1107,20 +1072,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBE57961-53EC-473A-96A6-73C5868578EB}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.7109375" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1128,315 +1092,272 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
         <v>0</v>
       </c>
-      <c r="I1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>73257316</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D12" t="s">
         <v>5</v>
       </c>
-      <c r="F2">
-        <v>5</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>72758956</v>
-      </c>
-      <c r="E3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="H3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>70477743</v>
-      </c>
-      <c r="E4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4">
-        <v>4</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>48344037</v>
-      </c>
-      <c r="E5" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>76586998</v>
-      </c>
-      <c r="E6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6">
-        <v>5</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>44883074</v>
-      </c>
-      <c r="E7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>4</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="H7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" t="s">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>72413556</v>
-      </c>
-      <c r="E8" t="s">
-        <v>5</v>
-      </c>
-      <c r="F8">
-        <v>5</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="H8" t="s">
-        <v>50</v>
-      </c>
-      <c r="I8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" t="s">
-        <v>1</v>
-      </c>
-      <c r="D9">
-        <v>72512391</v>
-      </c>
-      <c r="E9" t="s">
-        <v>5</v>
-      </c>
-      <c r="F9">
-        <v>4</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="H9" t="s">
-        <v>50</v>
-      </c>
-      <c r="I9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" t="s">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>70876605</v>
-      </c>
-      <c r="E10" t="s">
-        <v>5</v>
-      </c>
-      <c r="F10">
-        <v>5</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10" t="s">
-        <v>50</v>
-      </c>
-      <c r="I10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D11">
-        <v>72373931</v>
-      </c>
-      <c r="E11" t="s">
-        <v>5</v>
-      </c>
-      <c r="F11">
+      <c r="E12" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H11" t="s">
-        <v>50</v>
-      </c>
-      <c r="I11">
-        <v>2</v>
+      <c r="G12">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1450,20 +1371,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4357903D-29A3-4525-A3FB-868C7DC1FA3C}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.85546875" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1471,195 +1390,156 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>64</v>
       </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
         <v>5</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
         <v>11</v>
       </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>10762187</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
         <v>5</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>10</v>
-      </c>
-      <c r="H3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>72839865</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="E5">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
         <v>5</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>24</v>
-      </c>
-      <c r="H4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>74626735</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="E6">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
         <v>5</v>
       </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>25</v>
-      </c>
-      <c r="H5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="E7">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
         <v>49</v>
       </c>
-      <c r="C6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>72512391</v>
-      </c>
-      <c r="E6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>13</v>
-      </c>
-      <c r="H6" t="s">
-        <v>50</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>72413556</v>
-      </c>
-      <c r="E7" t="s">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
       <c r="G7">
-        <v>13</v>
-      </c>
-      <c r="H7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I7">
         <v>1</v>
       </c>
     </row>
@@ -1709,7 +1589,7 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2">
         <v>46461021</v>
@@ -1718,7 +1598,7 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
         <v>9</v>
@@ -1729,7 +1609,7 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3">
         <v>73257316</v>
@@ -1738,7 +1618,7 @@
         <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>
@@ -1749,7 +1629,7 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4">
         <v>47690367</v>
@@ -1758,7 +1638,7 @@
         <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F4" t="s">
         <v>11</v>
@@ -1790,7 +1670,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D1" t="s">
         <v>8</v>
@@ -1807,7 +1687,7 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
@@ -1816,7 +1696,7 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
         <v>12</v>
@@ -1827,16 +1707,16 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
         <v>9</v>
@@ -1847,7 +1727,7 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4" t="s">
         <v>1</v>
@@ -1856,10 +1736,10 @@
         <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1877,47 +1757,47 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -1925,47 +1805,47 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>